<commit_message>
use original file from Ale
</commit_message>
<xml_diff>
--- a/api/templates/tb_workload_summary/en.xlsx
+++ b/api/templates/tb_workload_summary/en.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25225"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect-2\api\templates\tb_workload_summary\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mah_a\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{97981C7E-AD23-4632-9520-7956B77B62E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192" tabRatio="815"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monthly" sheetId="1" r:id="rId1"/>
@@ -59,7 +60,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -268,7 +269,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -605,7 +606,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B18"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
@@ -699,7 +700,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B18"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
@@ -787,7 +788,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B18"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>

<commit_message>
- scope new report to all countries - try read template from country folder
</commit_message>
<xml_diff>
--- a/api/templates/tb_workload_summary/en.xlsx
+++ b/api/templates/tb_workload_summary/en.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25225"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mah_a\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect-2\api\templates\tb_workload_summary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97981C7E-AD23-4632-9520-7956B77B62E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192" tabRatio="815"/>
   </bookViews>
   <sheets>
     <sheet name="Monthly" sheetId="1" r:id="rId1"/>
@@ -45,9 +44,6 @@
     <t>MTB+</t>
   </si>
   <si>
-    <t>Province</t>
-  </si>
-  <si>
     <t>TB Workload Summary - by Month</t>
   </si>
   <si>
@@ -55,12 +51,15 @@
   </si>
   <si>
     <t>TB Workload Summary by Year</t>
+  </si>
+  <si>
+    <t>State</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -269,7 +268,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -606,7 +605,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B18"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
@@ -615,7 +614,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -636,7 +635,7 @@
     </row>
     <row r="5" spans="1:2" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -659,7 +658,7 @@
     </row>
     <row r="11" spans="1:2" s="1" customFormat="1" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.3">
@@ -685,7 +684,7 @@
     </row>
     <row r="17" spans="1:1" s="1" customFormat="1" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:1" s="1" customFormat="1" x14ac:dyDescent="0.3">
@@ -700,7 +699,95 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="31.796875" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="11" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="A1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B15" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B18"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
@@ -728,7 +815,7 @@
     </row>
     <row r="5" spans="1:2" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -751,7 +838,7 @@
     </row>
     <row r="11" spans="1:2" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
@@ -774,95 +861,7 @@
     </row>
     <row r="17" spans="1:1" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="31.796875" style="1" customWidth="1"/>
-    <col min="2" max="16384" width="11" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="2" t="s">
         <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B9" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B15" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="3" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.3">

</xml_diff>